<commit_message>
fix a major bug for refed state, where glycerol and blood linoleate substrate should be separated instead of shared
</commit_message>
<xml_diff>
--- a/CI compiled.xlsx
+++ b/CI compiled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/boyuan/Desktop/Harvard/Research/Energy Metabolism Atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3D8CC1-69B3-5A4E-A62F-BA10AA630E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E58678F0-042B-844D-AD95-0B0F6BF9D571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="22340" windowWidth="30240" windowHeight="18900" activeTab="4" xr2:uid="{C27F82BD-D1C2-DF4B-9AB6-A06FDDA3A96C}"/>
+    <workbookView xWindow="4080" yWindow="22360" windowWidth="30240" windowHeight="17280" activeTab="1" xr2:uid="{C27F82BD-D1C2-DF4B-9AB6-A06FDDA3A96C}"/>
   </bookViews>
   <sheets>
     <sheet name="Fasted base " sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Refed TAGkinetics_portalAAs" sheetId="5" r:id="rId5"/>
     <sheet name="flux_size" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -429,7 +429,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -688,7 +688,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -756,18 +756,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -782,13 +775,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -805,9 +792,6 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -832,18 +816,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -889,7 +865,7 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -904,17 +880,32 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2188,23 +2179,23 @@
         <v>47</v>
       </c>
       <c r="H1" s="1"/>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="86" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="88" t="s">
         <v>109</v>
       </c>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="78" t="s">
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="Q1" s="79" t="s">
+      <c r="Q1" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="80" t="s">
+      <c r="R1" s="70" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2231,29 +2222,29 @@
         <v>7.55</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="38" t="s">
+      <c r="J2" s="87"/>
+      <c r="K2" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="L2" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="M2" s="38" t="s">
+      <c r="M2" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="N2" s="49" t="s">
+      <c r="N2" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="71" t="s">
+      <c r="O2" s="91"/>
+      <c r="P2" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="Q2" s="72">
-        <f>K3</f>
+      <c r="Q2" s="62">
+        <f t="shared" ref="Q2:R4" si="0">K3</f>
         <v>28.875</v>
       </c>
-      <c r="R2" s="73">
-        <f>L3</f>
+      <c r="R2" s="63">
+        <f t="shared" si="0"/>
         <v>2.25</v>
       </c>
     </row>
@@ -2283,34 +2274,34 @@
       <c r="I3" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="J3" s="54">
+      <c r="J3" s="48">
         <v>39</v>
       </c>
-      <c r="K3" s="44">
+      <c r="K3" s="40">
         <f>J3/J5*K5</f>
         <v>28.875</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="33">
         <f>K3/K5*L5</f>
         <v>2.25</v>
       </c>
-      <c r="M3" s="35">
+      <c r="M3" s="32">
         <f>K3/K5*M5</f>
         <v>21</v>
       </c>
-      <c r="N3" s="50">
+      <c r="N3" s="45">
         <f>M3/M5*N5</f>
         <v>2.25</v>
       </c>
-      <c r="P3" s="35" t="s">
+      <c r="P3" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="Q3" s="36">
-        <f>K4</f>
+      <c r="Q3" s="33">
+        <f t="shared" si="0"/>
         <v>57.75</v>
       </c>
-      <c r="R3" s="50">
-        <f>L4</f>
+      <c r="R3" s="45">
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
     </row>
@@ -2340,34 +2331,34 @@
       <c r="I4" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="54">
+      <c r="J4" s="48">
         <v>78</v>
       </c>
-      <c r="K4" s="44">
+      <c r="K4" s="40">
         <f>J4/J5*K5</f>
         <v>57.75</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="33">
         <f>K4/K5*L5</f>
         <v>4.5</v>
       </c>
-      <c r="M4" s="35">
+      <c r="M4" s="32">
         <f>K4/K5*M5</f>
         <v>42</v>
       </c>
-      <c r="N4" s="50">
+      <c r="N4" s="45">
         <f>M4/M5*N5</f>
         <v>4.5</v>
       </c>
-      <c r="P4" s="38" t="s">
+      <c r="P4" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="Q4" s="39">
-        <f>K5</f>
+      <c r="Q4" s="36">
+        <f t="shared" si="0"/>
         <v>77</v>
       </c>
-      <c r="R4" s="74">
-        <f>L5</f>
+      <c r="R4" s="64">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
@@ -2397,30 +2388,30 @@
       <c r="I5" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="55">
+      <c r="J5" s="49">
         <v>104</v>
       </c>
-      <c r="K5" s="56">
+      <c r="K5" s="50">
         <f>77</f>
         <v>77</v>
       </c>
-      <c r="L5" s="57">
+      <c r="L5" s="51">
         <v>6</v>
       </c>
-      <c r="M5" s="55">
+      <c r="M5" s="49">
         <v>56</v>
       </c>
-      <c r="N5" s="58">
+      <c r="N5" s="52">
         <v>6</v>
       </c>
-      <c r="P5" s="71" t="s">
+      <c r="P5" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="Q5" s="72">
+      <c r="Q5" s="62">
         <f>SUM(Q2:Q4) * 1/3</f>
         <v>54.541666666666664</v>
       </c>
-      <c r="R5" s="73">
+      <c r="R5" s="63">
         <f>SQRT(R2^2 + R3^2 + R4^2 ) * 1/3</f>
         <v>2.6100766272276377</v>
       </c>
@@ -2448,31 +2439,31 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="K6" s="52">
+      <c r="K6" s="46">
         <f>SUM(K3:K5)</f>
         <v>163.625</v>
       </c>
-      <c r="L6" s="52">
+      <c r="L6" s="46">
         <f>SQRT(L3^2 + L4^2 +L5^2)</f>
         <v>7.8302298816829126</v>
       </c>
-      <c r="M6" s="53">
+      <c r="M6" s="47">
         <f>SUM(M3:M5)</f>
         <v>119</v>
       </c>
-      <c r="N6" s="52">
+      <c r="N6" s="46">
         <f>SQRT(N3^2 + N4^2 +N5^2)</f>
         <v>7.8302298816829126</v>
       </c>
-      <c r="P6" s="71" t="s">
+      <c r="P6" s="61" t="s">
         <v>119</v>
       </c>
-      <c r="Q6" s="75">
-        <f>M3</f>
+      <c r="Q6" s="65">
+        <f t="shared" ref="Q6:R8" si="1">M3</f>
         <v>21</v>
       </c>
-      <c r="R6" s="73">
-        <f>N3</f>
+      <c r="R6" s="63">
+        <f t="shared" si="1"/>
         <v>2.25</v>
       </c>
     </row>
@@ -2499,15 +2490,15 @@
         <v>2.35</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="P7" s="35" t="s">
+      <c r="P7" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="Q7" s="32">
-        <f>M4</f>
+      <c r="Q7" s="30">
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
-      <c r="R7" s="50">
-        <f>N4</f>
+      <c r="R7" s="45">
+        <f t="shared" si="1"/>
         <v>4.5</v>
       </c>
     </row>
@@ -2534,22 +2525,22 @@
         <v>1.45</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="K8" s="59"/>
-      <c r="L8" s="60" t="s">
+      <c r="K8" s="53"/>
+      <c r="L8" s="54" t="s">
         <v>101</v>
       </c>
-      <c r="M8" s="61" t="s">
+      <c r="M8" s="55" t="s">
         <v>102</v>
       </c>
-      <c r="P8" s="38" t="s">
+      <c r="P8" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="Q8" s="41">
-        <f>M5</f>
+      <c r="Q8" s="38">
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="R8" s="74">
-        <f>N5</f>
+      <c r="R8" s="64">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
@@ -2576,23 +2567,23 @@
         <v>1.5</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="K9" s="62" t="s">
+      <c r="K9" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="L9" s="63">
+      <c r="L9" s="57">
         <v>381</v>
       </c>
-      <c r="M9" s="64">
+      <c r="M9" s="58">
         <v>20</v>
       </c>
-      <c r="P9" s="38" t="s">
+      <c r="P9" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="Q9" s="39">
+      <c r="Q9" s="36">
         <f>SUM(Q6:Q8) * 1/3</f>
         <v>39.666666666666664</v>
       </c>
-      <c r="R9" s="74">
+      <c r="R9" s="64">
         <f>SQRT(R6^2 +R7^2 + R8^2 ) * 1/3</f>
         <v>2.6100766272276377</v>
       </c>
@@ -2620,23 +2611,23 @@
         <v>5.25</v>
       </c>
       <c r="H10" s="2"/>
-      <c r="K10" s="62" t="s">
+      <c r="K10" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="L10" s="63">
+      <c r="L10" s="57">
         <v>6</v>
       </c>
-      <c r="M10" s="64">
+      <c r="M10" s="58">
         <v>3</v>
       </c>
-      <c r="P10" s="45" t="s">
+      <c r="P10" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="Q10" s="69">
+      <c r="Q10" s="42">
         <f>L10</f>
         <v>6</v>
       </c>
-      <c r="R10" s="70">
+      <c r="R10" s="43">
         <f>M10</f>
         <v>3</v>
       </c>
@@ -2664,23 +2655,23 @@
         <v>5.25</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="K11" s="62" t="s">
+      <c r="K11" s="56" t="s">
         <v>104</v>
       </c>
-      <c r="L11" s="63">
+      <c r="L11" s="57">
         <v>32</v>
       </c>
-      <c r="M11" s="64">
+      <c r="M11" s="58">
         <v>4</v>
       </c>
-      <c r="P11" s="45" t="s">
+      <c r="P11" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="Q11" s="76">
+      <c r="Q11" s="66">
         <f>L12-SUM(Q2:Q9)-Q10</f>
         <v>62.166666666666686</v>
       </c>
-      <c r="R11" s="77">
+      <c r="R11" s="67">
         <f>SQRT(M12^2 + R2^2 + R3^2 + R4^2 +R6^2 +R7^2 +R8^2 + R5^2 + R9^2 +R10^2 )</f>
         <v>24.682990094394967</v>
       </c>
@@ -2708,14 +2699,14 @@
         <v>4.8499999999999996</v>
       </c>
       <c r="H12" s="2"/>
-      <c r="K12" s="68" t="s">
+      <c r="K12" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="L12" s="33">
+      <c r="L12">
         <f>L9+L11*2</f>
         <v>445</v>
       </c>
-      <c r="M12" s="34">
+      <c r="M12" s="31">
         <f>SQRT(M9^2+4*M11^2)</f>
         <v>21.540659228538015</v>
       </c>
@@ -2743,14 +2734,14 @@
         <v>3.4</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="K13" s="65" t="s">
+      <c r="K13" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="L13" s="40">
+      <c r="L13" s="37">
         <f>L12-L10-K6-M6</f>
         <v>156.375</v>
       </c>
-      <c r="M13" s="42">
+      <c r="M13" s="39">
         <f>SQRT(M12^2 + M10^2 + L6^2 + N6^2 )</f>
         <v>24.405429723731562</v>
       </c>
@@ -3805,13 +3796,13 @@
       <c r="B18" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="C18" s="81" t="s">
+      <c r="C18" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="82">
+      <c r="D18" s="72">
         <v>68.400000000000006</v>
       </c>
-      <c r="E18" s="82">
+      <c r="E18" s="72">
         <v>12.13232</v>
       </c>
       <c r="F18" s="12">
@@ -4254,23 +4245,23 @@
       <c r="G1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="86" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="88" t="s">
         <v>109</v>
       </c>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="78" t="s">
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="Q1" s="79" t="s">
+      <c r="Q1" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="80" t="s">
+      <c r="R1" s="70" t="s">
         <v>3</v>
       </c>
     </row>
@@ -4296,29 +4287,29 @@
       <c r="G2" s="10">
         <v>1.05</v>
       </c>
-      <c r="J2" s="43"/>
-      <c r="K2" s="38" t="s">
+      <c r="J2" s="87"/>
+      <c r="K2" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="L2" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="M2" s="38" t="s">
+      <c r="M2" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="N2" s="49" t="s">
+      <c r="N2" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="71" t="s">
+      <c r="O2" s="91"/>
+      <c r="P2" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="Q2" s="72">
-        <f>K3</f>
+      <c r="Q2" s="62">
+        <f t="shared" ref="Q2:R4" si="0">K3</f>
         <v>4.125</v>
       </c>
-      <c r="R2" s="73">
-        <f>L3</f>
+      <c r="R2" s="63">
+        <f t="shared" si="0"/>
         <v>1.875</v>
       </c>
     </row>
@@ -4347,34 +4338,34 @@
       <c r="I3" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="J3" s="88">
+      <c r="J3" s="78">
         <v>39</v>
       </c>
-      <c r="K3" s="44">
+      <c r="K3" s="40">
         <f>J3/J5*K5</f>
         <v>4.125</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="33">
         <f>K3/K5*L5</f>
         <v>1.875</v>
       </c>
-      <c r="M3" s="44">
+      <c r="M3" s="40">
         <f>K3/K5*M5</f>
         <v>20.25</v>
       </c>
-      <c r="N3" s="50">
+      <c r="N3" s="45">
         <f>M3/M5*N5</f>
         <v>3.375</v>
       </c>
-      <c r="P3" s="35" t="s">
+      <c r="P3" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="Q3" s="36">
-        <f>K4</f>
+      <c r="Q3" s="33">
+        <f t="shared" si="0"/>
         <v>8.25</v>
       </c>
-      <c r="R3" s="50">
-        <f>L4</f>
+      <c r="R3" s="45">
+        <f t="shared" si="0"/>
         <v>3.75</v>
       </c>
     </row>
@@ -4403,34 +4394,34 @@
       <c r="I4" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="88">
+      <c r="J4" s="78">
         <v>78</v>
       </c>
-      <c r="K4" s="44">
+      <c r="K4" s="40">
         <f>J4/J5*K5</f>
         <v>8.25</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="33">
         <f>K4/K5*L5</f>
         <v>3.75</v>
       </c>
-      <c r="M4" s="44">
+      <c r="M4" s="40">
         <f>K4/K5*M5</f>
         <v>40.5</v>
       </c>
-      <c r="N4" s="50">
+      <c r="N4" s="45">
         <f>M4/M5*N5</f>
         <v>6.75</v>
       </c>
-      <c r="P4" s="38" t="s">
+      <c r="P4" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="Q4" s="39">
-        <f>K5</f>
+      <c r="Q4" s="36">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="R4" s="74">
-        <f>L5</f>
+      <c r="R4" s="64">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
@@ -4459,29 +4450,29 @@
       <c r="I5" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="89">
+      <c r="J5" s="79">
         <v>104</v>
       </c>
-      <c r="K5" s="83">
+      <c r="K5" s="73">
         <v>11</v>
       </c>
-      <c r="L5" s="84">
+      <c r="L5" s="74">
         <v>5</v>
       </c>
-      <c r="M5" s="83">
+      <c r="M5" s="73">
         <v>54</v>
       </c>
-      <c r="N5" s="85">
+      <c r="N5" s="75">
         <v>9</v>
       </c>
-      <c r="P5" s="71" t="s">
+      <c r="P5" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="Q5" s="72">
+      <c r="Q5" s="62">
         <f>SUM(Q2:Q4) * 1/3</f>
         <v>7.791666666666667</v>
       </c>
-      <c r="R5" s="73">
+      <c r="R5" s="63">
         <f>SQRT(R2^2 + R3^2 + R4^2 ) * 1/3</f>
         <v>2.1750638560230313</v>
       </c>
@@ -4508,31 +4499,31 @@
       <c r="G6" s="10">
         <v>5.25</v>
       </c>
-      <c r="K6" s="52">
+      <c r="K6" s="46">
         <f>SUM(K3:K5)</f>
         <v>23.375</v>
       </c>
-      <c r="L6" s="52">
+      <c r="L6" s="46">
         <f>SQRT(L3^2 + L4^2 +L5^2)</f>
         <v>6.5251915680690935</v>
       </c>
-      <c r="M6" s="53">
+      <c r="M6" s="47">
         <f>SUM(M3:M5)</f>
         <v>114.75</v>
       </c>
-      <c r="N6" s="52">
+      <c r="N6" s="46">
         <f>SQRT(N3^2 + N4^2 +N5^2)</f>
         <v>11.74534482252437</v>
       </c>
-      <c r="P6" s="71" t="s">
+      <c r="P6" s="61" t="s">
         <v>119</v>
       </c>
-      <c r="Q6" s="75">
-        <f>M3</f>
+      <c r="Q6" s="65">
+        <f t="shared" ref="Q6:R8" si="1">M3</f>
         <v>20.25</v>
       </c>
-      <c r="R6" s="73">
-        <f>N3</f>
+      <c r="R6" s="63">
+        <f t="shared" si="1"/>
         <v>3.375</v>
       </c>
     </row>
@@ -4558,15 +4549,15 @@
       <c r="G7" s="10">
         <v>18.3</v>
       </c>
-      <c r="P7" s="35" t="s">
+      <c r="P7" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="Q7" s="32">
-        <f>M4</f>
+      <c r="Q7" s="30">
+        <f t="shared" si="1"/>
         <v>40.5</v>
       </c>
-      <c r="R7" s="50">
-        <f>N4</f>
+      <c r="R7" s="45">
+        <f t="shared" si="1"/>
         <v>6.75</v>
       </c>
     </row>
@@ -4592,22 +4583,22 @@
       <c r="G8" s="10">
         <v>96.1</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="60" t="s">
+      <c r="K8" s="53"/>
+      <c r="L8" s="54" t="s">
         <v>101</v>
       </c>
-      <c r="M8" s="61" t="s">
+      <c r="M8" s="55" t="s">
         <v>102</v>
       </c>
-      <c r="P8" s="38" t="s">
+      <c r="P8" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="Q8" s="41">
-        <f>M5</f>
+      <c r="Q8" s="38">
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
-      <c r="R8" s="74">
-        <f>N5</f>
+      <c r="R8" s="64">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -4633,23 +4624,23 @@
       <c r="G9" s="10">
         <v>111.05</v>
       </c>
-      <c r="K9" s="62" t="s">
+      <c r="K9" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="L9" s="86">
+      <c r="L9" s="76">
         <v>524</v>
       </c>
-      <c r="M9" s="87">
+      <c r="M9" s="77">
         <v>47</v>
       </c>
-      <c r="P9" s="38" t="s">
+      <c r="P9" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="Q9" s="39">
+      <c r="Q9" s="36">
         <f>SUM(Q6:Q8) * 1/3</f>
         <v>38.25</v>
       </c>
-      <c r="R9" s="74">
+      <c r="R9" s="64">
         <f>SQRT(R6^2 +R7^2 + R8^2 ) * 1/3</f>
         <v>3.9151149408414567</v>
       </c>
@@ -4676,23 +4667,23 @@
       <c r="G10" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="K10" s="62" t="s">
+      <c r="K10" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="L10" s="86">
+      <c r="L10" s="76">
         <v>31</v>
       </c>
-      <c r="M10" s="87">
+      <c r="M10" s="77">
         <v>6</v>
       </c>
-      <c r="P10" s="45" t="s">
+      <c r="P10" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="Q10" s="69">
+      <c r="Q10" s="42">
         <f>L10</f>
         <v>31</v>
       </c>
-      <c r="R10" s="70">
+      <c r="R10" s="43">
         <f>M10</f>
         <v>6</v>
       </c>
@@ -4719,23 +4710,23 @@
       <c r="G11" s="10">
         <v>111.85</v>
       </c>
-      <c r="K11" s="62" t="s">
+      <c r="K11" s="56" t="s">
         <v>104</v>
       </c>
-      <c r="L11" s="86">
+      <c r="L11" s="76">
         <v>10</v>
       </c>
-      <c r="M11" s="87">
+      <c r="M11" s="77">
         <v>2</v>
       </c>
-      <c r="P11" s="45" t="s">
+      <c r="P11" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="Q11" s="76">
+      <c r="Q11" s="66">
         <f>L12-SUM(Q2:Q9)-Q10</f>
         <v>328.83333333333331</v>
       </c>
-      <c r="R11" s="77">
+      <c r="R11" s="67">
         <f>SQRT(M12^2 + R2^2 + R3^2 + R4^2 +R6^2 +R7^2 +R8^2 + R5^2 + R9^2 +R10^2 )</f>
         <v>49.614416027781459</v>
       </c>
@@ -4762,14 +4753,14 @@
       <c r="G12" s="10">
         <v>0.8</v>
       </c>
-      <c r="K12" s="68" t="s">
+      <c r="K12" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="L12" s="33">
+      <c r="L12">
         <f>L9+L11*2</f>
         <v>544</v>
       </c>
-      <c r="M12" s="37">
+      <c r="M12" s="34">
         <f>SQRT(M9^2+4*M11^2)</f>
         <v>47.169905660283021</v>
       </c>
@@ -4796,14 +4787,14 @@
       <c r="G13" s="10">
         <v>1.1499999999999999</v>
       </c>
-      <c r="K13" s="65" t="s">
+      <c r="K13" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="L13" s="40">
+      <c r="L13" s="37">
         <f>L12-L10-K6-M6</f>
         <v>374.875</v>
       </c>
-      <c r="M13" s="66">
+      <c r="M13" s="60">
         <f>SQRT(M12^2 + M10^2 + L6^2 + N6^2 )</f>
         <v>49.411853335004544</v>
       </c>
@@ -5407,32 +5398,32 @@
       <c r="G1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="86" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="88" t="s">
         <v>109</v>
       </c>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="94" t="s">
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="83" t="s">
         <v>111</v>
       </c>
-      <c r="Q1" s="94" t="s">
+      <c r="Q1" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="94" t="s">
+      <c r="R1" s="83" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="94" t="s">
+      <c r="T1" s="83" t="s">
         <v>111</v>
       </c>
-      <c r="U1" s="94" t="s">
+      <c r="U1" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="V1" s="94" t="s">
+      <c r="V1" s="83" t="s">
         <v>3</v>
       </c>
     </row>
@@ -5458,41 +5449,41 @@
       <c r="G2" s="2">
         <v>2.1</v>
       </c>
-      <c r="J2" s="43"/>
-      <c r="K2" s="38" t="s">
+      <c r="J2" s="87"/>
+      <c r="K2" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="L2" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="M2" s="38" t="s">
+      <c r="M2" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="N2" s="49" t="s">
+      <c r="N2" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="91" t="s">
+      <c r="O2" s="91"/>
+      <c r="P2" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="Q2" s="92">
-        <f>K3</f>
+      <c r="Q2" s="82">
+        <f t="shared" ref="Q2:R4" si="0">K3</f>
         <v>5.25</v>
       </c>
-      <c r="R2" s="92">
-        <f>L3</f>
+      <c r="R2" s="82">
+        <f t="shared" si="0"/>
         <v>2.625</v>
       </c>
-      <c r="T2" s="91" t="str">
+      <c r="T2" s="81" t="str">
         <f>P2</f>
         <v>NEFA-Palm</v>
       </c>
-      <c r="U2" s="95">
-        <f t="shared" ref="U2:V2" si="0">Q2</f>
+      <c r="U2" s="84">
+        <f t="shared" ref="U2:V2" si="1">Q2</f>
         <v>5.25</v>
       </c>
-      <c r="V2" s="95">
-        <f t="shared" si="0"/>
+      <c r="V2" s="84">
+        <f t="shared" si="1"/>
         <v>2.625</v>
       </c>
     </row>
@@ -5521,51 +5512,51 @@
       <c r="I3" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="J3" s="88">
+      <c r="J3" s="78">
         <v>39</v>
       </c>
-      <c r="K3" s="44">
+      <c r="K3" s="40">
         <f>J3/J5*K5</f>
         <v>5.25</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="33">
         <f>K3/K5*L5</f>
         <v>2.625</v>
       </c>
-      <c r="M3" s="44">
+      <c r="M3" s="40">
         <f>K3/K5*M5</f>
         <v>21</v>
       </c>
-      <c r="N3" s="50">
+      <c r="N3" s="45">
         <f>M3/M5*N5</f>
         <v>3.375</v>
       </c>
-      <c r="P3" s="91" t="s">
+      <c r="P3" s="81" t="s">
         <v>117</v>
       </c>
-      <c r="Q3" s="92">
-        <f>K4</f>
+      <c r="Q3" s="82">
+        <f t="shared" si="0"/>
         <v>10.5</v>
       </c>
-      <c r="R3" s="92">
-        <f>L4</f>
+      <c r="R3" s="82">
+        <f t="shared" si="0"/>
         <v>5.25</v>
       </c>
-      <c r="T3" s="91" t="str">
-        <f t="shared" ref="T3:T4" si="1">P3</f>
+      <c r="T3" s="81" t="str">
+        <f t="shared" ref="T3:T4" si="2">P3</f>
         <v>NEFA-Ole</v>
       </c>
-      <c r="U3" s="95">
-        <f t="shared" ref="U3:U4" si="2">Q3</f>
+      <c r="U3" s="84">
+        <f t="shared" ref="U3:U4" si="3">Q3</f>
         <v>10.5</v>
       </c>
-      <c r="V3" s="95">
-        <f t="shared" ref="V3:V4" si="3">R3</f>
+      <c r="V3" s="84">
+        <f t="shared" ref="V3:V4" si="4">R3</f>
         <v>5.25</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A4" s="90">
+      <c r="A4" s="80">
         <v>3</v>
       </c>
       <c r="B4" s="7">
@@ -5589,51 +5580,51 @@
       <c r="I4" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="J4" s="88">
+      <c r="J4" s="78">
         <v>78</v>
       </c>
-      <c r="K4" s="44">
+      <c r="K4" s="40">
         <f>J4/J5*K5</f>
         <v>10.5</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="33">
         <f>K4/K5*L5</f>
         <v>5.25</v>
       </c>
-      <c r="M4" s="44">
+      <c r="M4" s="40">
         <f>K4/K5*M5</f>
         <v>42</v>
       </c>
-      <c r="N4" s="50">
+      <c r="N4" s="45">
         <f>M4/M5*N5</f>
         <v>6.75</v>
       </c>
-      <c r="P4" s="91" t="s">
+      <c r="P4" s="81" t="s">
         <v>118</v>
       </c>
-      <c r="Q4" s="92">
-        <f>K5</f>
+      <c r="Q4" s="82">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="R4" s="92">
-        <f>L5</f>
+      <c r="R4" s="82">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="T4" s="91" t="str">
-        <f t="shared" si="1"/>
+      <c r="T4" s="81" t="str">
+        <f t="shared" si="2"/>
         <v>NEFA-Lino</v>
       </c>
-      <c r="U4" s="95">
-        <f t="shared" si="2"/>
+      <c r="U4" s="84">
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="V4" s="95">
-        <f t="shared" si="3"/>
+      <c r="V4" s="84">
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="90">
+      <c r="A5" s="80">
         <v>4</v>
       </c>
       <c r="B5" s="7">
@@ -5657,47 +5648,47 @@
       <c r="I5" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="89">
+      <c r="J5" s="79">
         <v>104</v>
       </c>
-      <c r="K5" s="83">
+      <c r="K5" s="73">
         <v>14</v>
       </c>
-      <c r="L5" s="84">
+      <c r="L5" s="74">
         <v>7</v>
       </c>
-      <c r="M5" s="83">
+      <c r="M5" s="73">
         <v>56</v>
       </c>
-      <c r="N5" s="85">
+      <c r="N5" s="75">
         <v>9</v>
       </c>
-      <c r="P5" s="91" t="s">
+      <c r="P5" s="81" t="s">
         <v>113</v>
       </c>
-      <c r="Q5" s="92">
+      <c r="Q5" s="82">
         <f>SUM(Q2:Q4) * 1/3</f>
         <v>9.9166666666666661</v>
       </c>
-      <c r="R5" s="92">
+      <c r="R5" s="82">
         <f>SQRT(R2^2 + R3^2 + R4^2 ) * 1/3</f>
         <v>3.045089398432244</v>
       </c>
-      <c r="T5" s="91" t="str">
+      <c r="T5" s="81" t="str">
         <f>P6</f>
         <v>TAG-Palm</v>
       </c>
-      <c r="U5" s="95">
-        <f t="shared" ref="U5:U7" si="4">Q6</f>
+      <c r="U5" s="84">
+        <f t="shared" ref="U5:U7" si="5">Q6</f>
         <v>21</v>
       </c>
-      <c r="V5" s="95">
-        <f t="shared" ref="V5:V7" si="5">R6</f>
+      <c r="V5" s="84">
+        <f t="shared" ref="V5:V7" si="6">R6</f>
         <v>3.375</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A6" s="90">
+      <c r="A6" s="80">
         <v>5</v>
       </c>
       <c r="B6" s="7">
@@ -5718,48 +5709,48 @@
       <c r="G6" s="2">
         <v>11.4</v>
       </c>
-      <c r="K6" s="52">
+      <c r="K6" s="46">
         <f>SUM(K3:K5)</f>
         <v>29.75</v>
       </c>
-      <c r="L6" s="52">
+      <c r="L6" s="46">
         <f>SQRT(L3^2 + L4^2 +L5^2)</f>
         <v>9.1352681952967316</v>
       </c>
-      <c r="M6" s="53">
+      <c r="M6" s="47">
         <f>SUM(M3:M5)</f>
         <v>119</v>
       </c>
-      <c r="N6" s="52">
+      <c r="N6" s="46">
         <f>SQRT(N3^2 + N4^2 +N5^2)</f>
         <v>11.74534482252437</v>
       </c>
-      <c r="P6" s="91" t="s">
+      <c r="P6" s="81" t="s">
         <v>119</v>
       </c>
-      <c r="Q6" s="91">
-        <f>M3</f>
+      <c r="Q6" s="81">
+        <f t="shared" ref="Q6:R8" si="7">M3</f>
         <v>21</v>
       </c>
-      <c r="R6" s="92">
-        <f>N3</f>
+      <c r="R6" s="82">
+        <f t="shared" si="7"/>
         <v>3.375</v>
       </c>
-      <c r="T6" s="91" t="str">
+      <c r="T6" s="81" t="str">
         <f>P7</f>
         <v>TAG-Ole</v>
       </c>
-      <c r="U6" s="95">
-        <f t="shared" si="4"/>
+      <c r="U6" s="84">
+        <f t="shared" si="5"/>
         <v>42</v>
       </c>
-      <c r="V6" s="95">
-        <f t="shared" si="5"/>
+      <c r="V6" s="84">
+        <f t="shared" si="6"/>
         <v>6.75</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="90">
+      <c r="A7" s="80">
         <v>6</v>
       </c>
       <c r="B7" s="7">
@@ -5780,32 +5771,32 @@
       <c r="G7" s="2">
         <v>66.05</v>
       </c>
-      <c r="P7" s="91" t="s">
+      <c r="P7" s="81" t="s">
         <v>120</v>
       </c>
-      <c r="Q7" s="91">
-        <f>M4</f>
+      <c r="Q7" s="81">
+        <f t="shared" si="7"/>
         <v>42</v>
       </c>
-      <c r="R7" s="92">
-        <f>N4</f>
+      <c r="R7" s="82">
+        <f t="shared" si="7"/>
         <v>6.75</v>
       </c>
-      <c r="T7" s="91" t="str">
+      <c r="T7" s="81" t="str">
         <f>P8</f>
         <v>TAG-Lino</v>
       </c>
-      <c r="U7" s="95">
-        <f t="shared" si="4"/>
+      <c r="U7" s="84">
+        <f t="shared" si="5"/>
         <v>56</v>
       </c>
-      <c r="V7" s="95">
-        <f t="shared" si="5"/>
+      <c r="V7" s="84">
+        <f t="shared" si="6"/>
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A8" s="90">
+      <c r="A8" s="80">
         <v>7</v>
       </c>
       <c r="B8" s="7">
@@ -5826,39 +5817,39 @@
       <c r="G8" s="2">
         <v>920.9</v>
       </c>
-      <c r="K8" s="59"/>
-      <c r="L8" s="60" t="s">
+      <c r="K8" s="53"/>
+      <c r="L8" s="54" t="s">
         <v>101</v>
       </c>
-      <c r="M8" s="61" t="s">
+      <c r="M8" s="55" t="s">
         <v>102</v>
       </c>
-      <c r="P8" s="91" t="s">
+      <c r="P8" s="81" t="s">
         <v>121</v>
       </c>
-      <c r="Q8" s="91">
-        <f>M5</f>
+      <c r="Q8" s="81">
+        <f t="shared" si="7"/>
         <v>56</v>
       </c>
-      <c r="R8" s="92">
-        <f>N5</f>
+      <c r="R8" s="82">
+        <f t="shared" si="7"/>
         <v>9</v>
       </c>
-      <c r="T8" s="91" t="str">
-        <f>P10</f>
+      <c r="T8" s="81" t="str">
+        <f t="shared" ref="T8:V9" si="8">P10</f>
         <v>Amino Acids</v>
       </c>
-      <c r="U8" s="95">
-        <f>Q10</f>
+      <c r="U8" s="84">
+        <f t="shared" si="8"/>
         <v>163</v>
       </c>
-      <c r="V8" s="95">
-        <f>R10</f>
+      <c r="V8" s="84">
+        <f t="shared" si="8"/>
         <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A9" s="90">
+      <c r="A9" s="80">
         <v>8</v>
       </c>
       <c r="B9" s="7">
@@ -5879,41 +5870,41 @@
       <c r="G9" s="2">
         <v>986.8</v>
       </c>
-      <c r="K9" s="62" t="s">
+      <c r="K9" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="L9" s="86">
+      <c r="L9" s="76">
         <v>331</v>
       </c>
-      <c r="M9" s="87">
+      <c r="M9" s="77">
         <v>38</v>
       </c>
-      <c r="P9" s="91" t="s">
+      <c r="P9" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="Q9" s="92">
+      <c r="Q9" s="82">
         <f>SUM(Q6:Q8) * 1/3</f>
         <v>39.666666666666664</v>
       </c>
-      <c r="R9" s="92">
+      <c r="R9" s="82">
         <f>SQRT(R6^2 +R7^2 + R8^2 ) * 1/3</f>
         <v>3.9151149408414567</v>
       </c>
-      <c r="T9" s="91" t="str">
-        <f>P11</f>
+      <c r="T9" s="81" t="str">
+        <f t="shared" si="8"/>
         <v>carbs</v>
       </c>
-      <c r="U9" s="95">
-        <f>Q11</f>
+      <c r="U9" s="84">
+        <f t="shared" si="8"/>
         <v>32</v>
       </c>
-      <c r="V9" s="95">
-        <f>R11</f>
+      <c r="V9" s="84">
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A10" s="90">
+      <c r="A10" s="80">
         <v>9</v>
       </c>
       <c r="B10" s="7">
@@ -5934,41 +5925,41 @@
       <c r="G10" s="2">
         <v>3.95</v>
       </c>
-      <c r="K10" s="62" t="s">
+      <c r="K10" s="56" t="s">
         <v>104</v>
       </c>
-      <c r="L10" s="86">
+      <c r="L10" s="76">
         <v>12</v>
       </c>
-      <c r="M10" s="87">
+      <c r="M10" s="77">
         <v>2</v>
       </c>
-      <c r="P10" s="93" t="s">
+      <c r="P10" s="81" t="s">
         <v>124</v>
       </c>
-      <c r="Q10" s="91">
+      <c r="Q10" s="81">
         <f>L12</f>
         <v>163</v>
       </c>
-      <c r="R10" s="91">
+      <c r="R10" s="81">
         <f>M12</f>
         <v>50</v>
       </c>
-      <c r="T10" s="91" t="str">
+      <c r="T10" s="81" t="str">
         <f>P12</f>
         <v>others</v>
       </c>
-      <c r="U10" s="95">
+      <c r="U10" s="84">
         <f>L13- SUM(U2:U9)</f>
         <v>11.25</v>
       </c>
-      <c r="V10" s="95">
+      <c r="V10" s="84">
         <f>R12</f>
         <v>65.046190852689023</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A11" s="90">
+      <c r="A11" s="80">
         <v>10</v>
       </c>
       <c r="B11" s="7">
@@ -5989,29 +5980,29 @@
       <c r="G11" s="2">
         <v>920</v>
       </c>
-      <c r="K11" s="62" t="s">
+      <c r="K11" s="56" t="s">
         <v>103</v>
       </c>
-      <c r="L11" s="86">
+      <c r="L11" s="76">
         <v>32</v>
       </c>
-      <c r="M11" s="87">
+      <c r="M11" s="77">
         <v>5</v>
       </c>
-      <c r="P11" s="91" t="s">
+      <c r="P11" s="81" t="s">
         <v>115</v>
       </c>
-      <c r="Q11" s="91">
+      <c r="Q11" s="81">
         <f>L11</f>
         <v>32</v>
       </c>
-      <c r="R11" s="91">
+      <c r="R11" s="81">
         <f>M11</f>
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A12" s="90">
+      <c r="A12" s="80">
         <v>11</v>
       </c>
       <c r="B12" s="7">
@@ -6032,29 +6023,29 @@
       <c r="G12" s="2">
         <v>1.2</v>
       </c>
-      <c r="K12" s="67" t="s">
+      <c r="K12" t="s">
         <v>123</v>
       </c>
-      <c r="L12" s="86">
+      <c r="L12" s="76">
         <v>163</v>
       </c>
-      <c r="M12" s="86">
+      <c r="M12" s="76">
         <v>50</v>
       </c>
-      <c r="P12" s="91" t="s">
+      <c r="P12" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="Q12" s="92">
+      <c r="Q12" s="82">
         <f>L13-SUM(Q2:Q9)-Q11-Q10</f>
         <v>-38.333333333333314</v>
       </c>
-      <c r="R12" s="92">
+      <c r="R12" s="82">
         <f>SQRT(M13^2 + R2^2 + R3^2 + R4^2 +R6^2 +R7^2 +R8^2 + R5^2 + R9^2 +R11^2  + R10^2)</f>
         <v>65.046190852689023</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A13" s="90">
+      <c r="A13" s="80">
         <v>12</v>
       </c>
       <c r="B13" s="7">
@@ -6075,26 +6066,26 @@
       <c r="G13" s="2">
         <v>2.15</v>
       </c>
-      <c r="K13" s="68" t="s">
+      <c r="K13" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="L13" s="33">
+      <c r="L13">
         <f>L9+L10*2</f>
         <v>355</v>
       </c>
-      <c r="M13" s="37">
+      <c r="M13" s="34">
         <f>SQRT(M9^2+4*M10^2)</f>
         <v>38.209946349085598</v>
       </c>
-      <c r="P13" s="96" t="s">
+      <c r="P13" s="85" t="s">
         <v>125</v>
       </c>
-      <c r="T13" s="96" t="s">
+      <c r="T13" s="85" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="90">
+      <c r="A14" s="80">
         <v>13</v>
       </c>
       <c r="B14" s="7">
@@ -6115,20 +6106,20 @@
       <c r="G14" s="2">
         <v>1.65</v>
       </c>
-      <c r="K14" s="65" t="s">
+      <c r="K14" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="L14" s="40">
+      <c r="L14" s="37">
         <f>L13-L11-K6-M6-L12</f>
         <v>11.25</v>
       </c>
-      <c r="M14" s="66">
+      <c r="M14" s="60">
         <f>SQRT(M13^2 + M11^2 + L6^2 + N6^2 + M12^2 )</f>
         <v>64.856813443153371</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A15" s="90">
+      <c r="A15" s="80">
         <v>14</v>
       </c>
       <c r="B15" s="7">
@@ -6151,7 +6142,7 @@
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A16" s="90">
+      <c r="A16" s="80">
         <v>15</v>
       </c>
       <c r="B16" s="7">
@@ -6174,7 +6165,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="90">
+      <c r="A17" s="80">
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
@@ -6197,7 +6188,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="90">
+      <c r="A18" s="80">
         <v>17</v>
       </c>
       <c r="B18" s="7">
@@ -6220,7 +6211,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="90">
+      <c r="A19" s="80">
         <v>18</v>
       </c>
       <c r="B19" s="7">
@@ -6243,7 +6234,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="90">
+      <c r="A20" s="80">
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
@@ -6266,7 +6257,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="90">
+      <c r="A21" s="80">
         <v>20</v>
       </c>
       <c r="B21" s="7">
@@ -6289,7 +6280,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="90">
+      <c r="A22" s="80">
         <v>21</v>
       </c>
       <c r="B22" s="7">
@@ -6312,7 +6303,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="90">
+      <c r="A23" s="80">
         <v>22</v>
       </c>
       <c r="B23" s="7">
@@ -6335,7 +6326,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="90">
+      <c r="A24" s="80">
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
@@ -6358,7 +6349,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="90">
+      <c r="A25" s="80">
         <v>24</v>
       </c>
       <c r="B25" s="7">
@@ -6381,7 +6372,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="90">
+      <c r="A26" s="80">
         <v>25</v>
       </c>
       <c r="B26" s="7">
@@ -6404,7 +6395,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="90">
+      <c r="A27" s="80">
         <v>26</v>
       </c>
       <c r="B27" s="7">
@@ -6427,7 +6418,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="90">
+      <c r="A28" s="80">
         <v>27</v>
       </c>
       <c r="B28" s="7">
@@ -6450,7 +6441,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="90">
+      <c r="A29" s="80">
         <v>28</v>
       </c>
       <c r="B29" s="7">
@@ -6473,7 +6464,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="90">
+      <c r="A30" s="80">
         <v>29</v>
       </c>
       <c r="B30" s="7">
@@ -6496,7 +6487,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="90">
+      <c r="A31" s="80">
         <v>30</v>
       </c>
       <c r="B31" s="7">
@@ -6519,7 +6510,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="90">
+      <c r="A32" s="80">
         <v>31</v>
       </c>
       <c r="B32" s="7">
@@ -6542,7 +6533,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="90">
+      <c r="A33" s="80">
         <v>32</v>
       </c>
       <c r="B33" s="7">
@@ -6565,7 +6556,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="90">
+      <c r="A34" s="80">
         <v>33</v>
       </c>
       <c r="B34" s="7">
@@ -6588,7 +6579,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="90">
+      <c r="A35" s="80">
         <v>34</v>
       </c>
       <c r="B35" s="7">
@@ -6611,7 +6602,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="90">
+      <c r="A36" s="80">
         <v>35</v>
       </c>
       <c r="B36" s="7" t="s">
@@ -6634,7 +6625,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="90">
+      <c r="A37" s="80">
         <v>36</v>
       </c>
       <c r="B37" s="7">
@@ -6657,7 +6648,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="90">
+      <c r="A38" s="80">
         <v>37</v>
       </c>
       <c r="B38" s="7">
@@ -6680,7 +6671,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="90">
+      <c r="A39" s="80">
         <v>38</v>
       </c>
       <c r="B39" s="7">
@@ -6703,7 +6694,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="90">
+      <c r="A40" s="80">
         <v>39</v>
       </c>
       <c r="B40" s="7">
@@ -6726,7 +6717,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="90">
+      <c r="A41" s="80">
         <v>40</v>
       </c>
       <c r="B41" s="7">
@@ -6749,7 +6740,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="90">
+      <c r="A42" s="80">
         <v>41</v>
       </c>
       <c r="B42" s="7">
@@ -6772,7 +6763,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="90">
+      <c r="A43" s="80">
         <v>42</v>
       </c>
       <c r="B43" s="7">
@@ -6795,7 +6786,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="90">
+      <c r="A44" s="80">
         <v>43</v>
       </c>
       <c r="B44" s="7">
@@ -6818,7 +6809,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="90">
+      <c r="A45" s="80">
         <v>44</v>
       </c>
       <c r="B45" s="7" t="s">
@@ -6841,7 +6832,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="90">
+      <c r="A46" s="80">
         <v>45</v>
       </c>
       <c r="B46" s="7">
@@ -6864,7 +6855,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="90">
+      <c r="A47" s="80">
         <v>46</v>
       </c>
       <c r="B47" s="7">
@@ -6887,7 +6878,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A48" s="90">
+      <c r="A48" s="80">
         <v>47</v>
       </c>
       <c r="B48" s="7">
@@ -6910,7 +6901,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="90">
+      <c r="A49" s="80">
         <v>48</v>
       </c>
       <c r="B49" s="7" t="s">
@@ -6933,7 +6924,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="90">
+      <c r="A50" s="80">
         <v>49</v>
       </c>
       <c r="B50" s="7">
@@ -6956,7 +6947,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51" s="90">
+      <c r="A51" s="80">
         <v>50</v>
       </c>
       <c r="B51" s="7">
@@ -6979,7 +6970,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52" s="90">
+      <c r="A52" s="80">
         <v>51</v>
       </c>
       <c r="B52" s="7">
@@ -7002,7 +6993,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A53" s="90">
+      <c r="A53" s="80">
         <v>52</v>
       </c>
       <c r="B53" s="7">
@@ -7025,7 +7016,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A54" s="90">
+      <c r="A54" s="80">
         <v>53</v>
       </c>
       <c r="B54" s="7">
@@ -7048,7 +7039,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="90">
+      <c r="A55" s="80">
         <v>54</v>
       </c>
       <c r="B55" s="7" t="s">
@@ -7071,7 +7062,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="90">
+      <c r="A56" s="80">
         <v>55</v>
       </c>
       <c r="B56" s="7">
@@ -7094,7 +7085,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="90">
+      <c r="A57" s="80">
         <v>56</v>
       </c>
       <c r="B57" s="7">
@@ -7117,7 +7108,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A58" s="90">
+      <c r="A58" s="80">
         <v>57</v>
       </c>
       <c r="B58" s="7">
@@ -7140,7 +7131,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A59" s="90">
+      <c r="A59" s="80">
         <v>58</v>
       </c>
       <c r="B59" s="7">
@@ -7163,7 +7154,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A60" s="90">
+      <c r="A60" s="80">
         <v>59</v>
       </c>
       <c r="B60" s="7">

</xml_diff>